<commit_message>
Update banner size and add MM-BASE USB parts
</commit_message>
<xml_diff>
--- a/modules/mm-base/bom/mm-base-gen1-reva-bom.xlsx
+++ b/modules/mm-base/bom/mm-base-gen1-reva-bom.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andre\Desktop\MakaniMotion\Engineering\mm-fan-gen1\mm-fan-gen1\modules\mm-base\bom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74B44809-978F-4F37-8504-6429F1CEAE17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0118F5F0-94A7-4C65-BEEA-9A8FB738B214}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{790FE4A5-72AF-4AEE-9175-50CBEDA28C41}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="80">
   <si>
     <t>Project</t>
   </si>
@@ -274,6 +274,24 @@
   </si>
   <si>
     <t>M3 x 6mm</t>
+  </si>
+  <si>
+    <t>USB C 180 Degree Angled Adapter</t>
+  </si>
+  <si>
+    <t>https://www.amazon.de/-/en/dp/B0BLMTGX8H?ref_=ppx_hzsearch_conn_dt_b_fed_asin_title_8&amp;th=1</t>
+  </si>
+  <si>
+    <t>buy</t>
+  </si>
+  <si>
+    <t>USB C Cable 0.5m</t>
+  </si>
+  <si>
+    <t>Depending on the USB connector, this adapter is necessary</t>
+  </si>
+  <si>
+    <t>Short cable for connecting a power bank</t>
   </si>
 </sst>
 </file>
@@ -751,13 +769,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF24B295-6732-4C2F-8811-9D8AD1EBF7D7}">
-  <dimension ref="A1:N28"/>
+  <dimension ref="A1:N30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
     <col min="2" max="2" width="41.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="62.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="47.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="53.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="32.7109375" customWidth="1"/>
     <col min="7" max="7" width="40.7109375" customWidth="1"/>
     <col min="8" max="8" width="13.42578125" style="8" bestFit="1" customWidth="1"/>
@@ -1240,6 +1258,43 @@
         <v>72</v>
       </c>
     </row>
+    <row r="29" spans="1:9">
+      <c r="A29" s="12">
+        <v>8</v>
+      </c>
+      <c r="B29" t="s">
+        <v>74</v>
+      </c>
+      <c r="D29" t="s">
+        <v>78</v>
+      </c>
+      <c r="E29">
+        <v>1</v>
+      </c>
+      <c r="F29" t="s">
+        <v>76</v>
+      </c>
+      <c r="I29" s="7" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9">
+      <c r="A30" s="12">
+        <v>9</v>
+      </c>
+      <c r="B30" t="s">
+        <v>77</v>
+      </c>
+      <c r="D30" t="s">
+        <v>79</v>
+      </c>
+      <c r="E30">
+        <v>1</v>
+      </c>
+      <c r="F30" t="s">
+        <v>76</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="I10" r:id="rId1" xr:uid="{6C6C2F25-B5AF-4A61-8404-204CD2581AD8}"/>
@@ -1253,9 +1308,10 @@
     <hyperlink ref="I18" r:id="rId9" xr:uid="{31F70C94-10E2-4175-B596-12C38D056058}"/>
     <hyperlink ref="I19" r:id="rId10" xr:uid="{1887D939-BA9F-433D-A8D5-6620265457C8}"/>
     <hyperlink ref="I27" r:id="rId11" xr:uid="{B399B27F-D581-4E0D-B68C-C03AAF0CF789}"/>
+    <hyperlink ref="I29" r:id="rId12" xr:uid="{36D750B2-C3C4-4659-ACAD-46E168A658B2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId12"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId13"/>
   <ignoredErrors>
     <ignoredError sqref="H15 H18" numberStoredAsText="1"/>
   </ignoredErrors>

</xml_diff>